<commit_message>
chore: anonymize client, operator, and database identifiers
Replace project and contractor names, personal accounts, and the
hardcoded database target with generic wording and schema names so
the plugin and SQL stay consistent without embedding client data.

Co-authored-by: Youcef ADDA <yadda07@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/files/template_dqe_exe.xlsx
+++ b/files/template_dqe_exe.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yadda\AppData\Roaming\QGIS\QGIS3\profiles\default\python\plugins\dqe_chargeur_marche_v3\files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\AppData\Roaming\QGIS\QGIS3\profiles\default\python\plugins\dqe_chargeur_marche_v3\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5110107-9A58-4E45-9810-B294378A528A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
@@ -389,7 +389,7 @@
     <t xml:space="preserve"> Pose de poteaux</t>
   </si>
   <si>
-    <t>pose poteau RAUV</t>
+    <t>pose poteau reseau</t>
   </si>
   <si>
     <t xml:space="preserve"> Fourniture des Alvéoles</t>

</xml_diff>

<commit_message>
chore: anonymize client, operator, and database identifiers (#1)
Replace project and contractor names, personal accounts, and the
hardcoded database target with generic wording and schema names so
the plugin and SQL stay consistent without embedding client data.

Co-authored-by: Cursor Agent <cursoragent@cursor.com>
Co-authored-by: Youcef ADDA <yadda07@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/files/template_dqe_exe.xlsx
+++ b/files/template_dqe_exe.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yadda\AppData\Roaming\QGIS\QGIS3\profiles\default\python\plugins\dqe_chargeur_marche_v3\files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\AppData\Roaming\QGIS\QGIS3\profiles\default\python\plugins\dqe_chargeur_marche_v3\files\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5110107-9A58-4E45-9810-B294378A528A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
@@ -389,7 +389,7 @@
     <t xml:space="preserve"> Pose de poteaux</t>
   </si>
   <si>
-    <t>pose poteau RAUV</t>
+    <t>pose poteau reseau</t>
   </si>
   <si>
     <t xml:space="preserve"> Fourniture des Alvéoles</t>

</xml_diff>